<commit_message>
Added new RDF data schemes and visual schemes for education-table13-17, fixed XLSX spreadsheets for education-table13-17
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table14.xlsx
+++ b/sources/table_normalization/xlsx/education-table14.xlsx
@@ -689,8 +689,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="#,##0.0"/>
-    <numFmt numFmtId="169" formatCode="\U\ \ \ #,##0.0;\U\ \ \ \-#,##0.0"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="\U\ \ \ #,##0.0;\U\ \ \ \-#,##0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -855,27 +855,14 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" readingOrder="1"/>
@@ -886,23 +873,36 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1186,154 +1186,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13">
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:13">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:13">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:13">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:13">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="30" customHeight="1">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="J10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="K10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="L10" s="16" t="s">
+      <c r="L10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M10" s="16" t="s">
+      <c r="M10" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="2:13">
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="K11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="M11" s="14" t="s">
+      <c r="C11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="M11" s="12" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="2:13" ht="15" customHeight="1">
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="9" t="s">
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="2:13" ht="15" customHeight="1">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="10"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="15"/>
     </row>
     <row r="14" spans="2:13">
       <c r="B14" s="1" t="s">
@@ -2324,38 +2324,38 @@
       </c>
     </row>
     <row r="40" spans="2:14" ht="15" customHeight="1">
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
-      <c r="K40" s="8"/>
-      <c r="L40" s="8"/>
-      <c r="M40" s="9" t="s">
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="41" spans="2:14" ht="15" customHeight="1">
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="10"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="18"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="15"/>
     </row>
     <row r="42" spans="2:14">
       <c r="B42" s="1" t="s">
@@ -2434,10 +2434,10 @@
       </c>
     </row>
     <row r="45" spans="2:14">
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="N45" s="6" t="s">
+      <c r="N45" s="13" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>